<commit_message>
ingesta: snapshot 2026-07-22 18:36 UTC
</commit_message>
<xml_diff>
--- a/data_lake/datos_diarios_preliminares/dt=2026-07-22/CORDOBA_JUL26.xlsx
+++ b/data_lake/datos_diarios_preliminares/dt=2026-07-22/CORDOBA_JUL26.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{030C547A-012E-4C73-811C-49A86E9FE4F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34B162B6-0779-461F-A049-1F44C5D560F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{5F8F14AC-D557-4126-B18A-7A2C1E69122F}"/>
   </bookViews>
@@ -7393,7 +7393,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -7866,7 +7866,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -8470,7 +8470,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -9079,7 +9079,7 @@
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -9689,7 +9689,7 @@
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-MX"/>
+  <c:lang val="es-ES"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -10020,7 +10020,7 @@
                   <c:v>36.799999999999997</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>-1</c:v>
+                  <c:v>2.4</c:v>
                 </c:pt>
                 <c:pt idx="21">
                   <c:v>-1</c:v>
@@ -19979,7 +19979,9 @@
       <c r="X3" s="25">
         <v>0</v>
       </c>
-      <c r="Y3" s="25"/>
+      <c r="Y3" s="25">
+        <v>0</v>
+      </c>
       <c r="Z3" s="25"/>
       <c r="AA3" s="25"/>
       <c r="AB3" s="25"/>
@@ -20071,7 +20073,9 @@
       <c r="X4" s="25">
         <v>1</v>
       </c>
-      <c r="Y4" s="25"/>
+      <c r="Y4" s="25">
+        <v>0</v>
+      </c>
       <c r="Z4" s="25"/>
       <c r="AA4" s="25"/>
       <c r="AB4" s="25"/>
@@ -20163,7 +20167,9 @@
       <c r="X5" s="25">
         <v>16.399999999999999</v>
       </c>
-      <c r="Y5" s="25"/>
+      <c r="Y5" s="25">
+        <v>0</v>
+      </c>
       <c r="Z5" s="25"/>
       <c r="AA5" s="25"/>
       <c r="AB5" s="25"/>
@@ -20255,7 +20261,9 @@
       <c r="X6" s="25">
         <v>4.7</v>
       </c>
-      <c r="Y6" s="25"/>
+      <c r="Y6" s="25">
+        <v>2.4</v>
+      </c>
       <c r="Z6" s="25"/>
       <c r="AA6" s="25"/>
       <c r="AB6" s="25"/>
@@ -20268,7 +20276,7 @@
       <c r="AI6" s="34"/>
       <c r="AJ6" s="36">
         <f t="shared" si="0"/>
-        <v>115.2</v>
+        <v>117.60000000000001</v>
       </c>
       <c r="AK6" s="30">
         <v>88.719230769230762</v>
@@ -20451,7 +20459,9 @@
       <c r="X9" s="25">
         <v>1</v>
       </c>
-      <c r="Y9" s="25"/>
+      <c r="Y9" s="25">
+        <v>0</v>
+      </c>
       <c r="Z9" s="25"/>
       <c r="AA9" s="25"/>
       <c r="AB9" s="25"/>
@@ -20619,7 +20629,9 @@
       <c r="X11" s="25">
         <v>0.4</v>
       </c>
-      <c r="Y11" s="25"/>
+      <c r="Y11" s="25">
+        <v>0</v>
+      </c>
       <c r="Z11" s="25"/>
       <c r="AA11" s="25"/>
       <c r="AB11" s="25"/>
@@ -20709,7 +20721,9 @@
       <c r="X12" s="25">
         <v>9.3000000000000007</v>
       </c>
-      <c r="Y12" s="25"/>
+      <c r="Y12" s="25">
+        <v>0</v>
+      </c>
       <c r="Z12" s="25"/>
       <c r="AA12" s="25"/>
       <c r="AB12" s="25"/>
@@ -20801,7 +20815,9 @@
       <c r="X13" s="25">
         <v>4</v>
       </c>
-      <c r="Y13" s="25"/>
+      <c r="Y13" s="25">
+        <v>0</v>
+      </c>
       <c r="Z13" s="25"/>
       <c r="AA13" s="25"/>
       <c r="AB13" s="25"/>
@@ -20891,7 +20907,9 @@
       <c r="X14" s="25">
         <v>0</v>
       </c>
-      <c r="Y14" s="25"/>
+      <c r="Y14" s="25">
+        <v>0</v>
+      </c>
       <c r="Z14" s="25"/>
       <c r="AA14" s="25"/>
       <c r="AB14" s="25"/>
@@ -20983,7 +21001,9 @@
       <c r="X15" s="25">
         <v>0</v>
       </c>
-      <c r="Y15" s="25"/>
+      <c r="Y15" s="25">
+        <v>0</v>
+      </c>
       <c r="Z15" s="25"/>
       <c r="AA15" s="25"/>
       <c r="AB15" s="25"/>
@@ -21186,7 +21206,7 @@
       </c>
       <c r="Y19" s="26">
         <f t="shared" si="1"/>
-        <v>-1</v>
+        <v>2.4</v>
       </c>
       <c r="Z19" s="26">
         <f t="shared" si="1"/>

</xml_diff>